<commit_message>
modification of test documents
</commit_message>
<xml_diff>
--- a/Test-Documentations/UI_Test_Execution_Reports/Signup Test Execution Reports.xlsx
+++ b/Test-Documentations/UI_Test_Execution_Reports/Signup Test Execution Reports.xlsx
@@ -5,16 +5,15 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="00_Project Overview" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="02_Valid Signup &amp; Field Validat" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="03_Password Rules" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="04_Profile Picture Upload Rules" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="05_Boundary Testing" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="06_Security Testing" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="07_UI Behavior and Submission C" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="01_Valid Signup &amp; Field Validat" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="02_Password Rules" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="03_Profile Picture Upload Rules" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="04_Boundary Testing" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="05_Security Testing" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="195">
   <si>
     <t xml:space="preserve">Project Overview</t>
   </si>
@@ -396,73 +395,67 @@
     <t xml:space="preserve">Password Above Maximum Length(26 characters)</t>
   </si>
   <si>
+    <t xml:space="preserve">Actual Result </t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valid Image Upload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image accepted. Stored with unique filename. Accessible via generated URL. No executable permission. Session established.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invalid File Type Upload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.exe and .pdf rejected correctly. No file stored. No account created.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Image Exceeding Size Limit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5MB file rejected. Proper validation message shown. No partial upload on server.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrupted Image Upload</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrupted image rejected</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC-024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renamed Executable File Upload</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">System accepted 22-character password. Validation missing for max length.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DEF-001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Actual Result </t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR-021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valid Image Upload</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Image accepted. Stored with unique filename. Accessible via generated URL. No executable permission. Session established.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR-022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Invalid File Type Upload</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.exe and .pdf rejected correctly. No file stored. No account created.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR-023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-022</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Image Exceeding Size Limit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.5MB file rejected. Proper validation message shown. No partial upload on server.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR-024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-023</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrupted Image Upload</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrupted image rejected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TR-025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC-024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renamed Executable File Upload</t>
   </si>
   <si>
     <t xml:space="preserve">Renamed .exe file (Malware.png) accepted. MIME validation missing. Security vulnerability confirmed.</t>
@@ -660,15 +653,6 @@
   </si>
   <si>
     <t xml:space="preserve">Input sanitized. No reflected or stored XSS observed. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seller Dashboard</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TC ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TS ID</t>
   </si>
 </sst>
 </file>
@@ -848,7 +832,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -978,10 +962,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2418,7 +2398,7 @@
       </c>
       <c r="J11" s="23"/>
     </row>
-    <row r="12" s="1" customFormat="true" ht="45.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="1" customFormat="true" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="29" t="s">
         <v>110</v>
       </c>
@@ -2437,159 +2417,159 @@
       <c r="F12" s="31" t="n">
         <v>46084</v>
       </c>
-      <c r="G12" s="33" t="s">
-        <v>113</v>
+      <c r="G12" s="32" t="s">
+        <v>35</v>
       </c>
       <c r="H12" s="29" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="I12" s="29" t="s">
-        <v>115</v>
+        <v>37</v>
       </c>
       <c r="J12" s="23"/>
     </row>
     <row r="13" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="37"/>
+      <c r="A13" s="33"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="36"/>
     </row>
     <row r="14" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="37"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="33"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="36"/>
     </row>
     <row r="15" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="37"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="36"/>
     </row>
     <row r="16" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="37"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="36"/>
     </row>
     <row r="17" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="37"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="36"/>
     </row>
     <row r="18" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="37"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="36"/>
     </row>
     <row r="19" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="37"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="36"/>
     </row>
     <row r="20" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="37"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="36"/>
     </row>
     <row r="21" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="37"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="36"/>
     </row>
     <row r="22" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="37"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="36"/>
     </row>
     <row r="23" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="37"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="36"/>
     </row>
     <row r="24" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="37"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="36"/>
     </row>
     <row r="25" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="37"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="36"/>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -2680,31 +2660,31 @@
       <c r="C5" s="15"/>
     </row>
     <row r="7" customFormat="false" ht="24.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="39" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="40" t="s">
+      <c r="C7" s="39" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="39" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="40" t="s">
+      <c r="G7" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="40" t="s">
-        <v>116</v>
-      </c>
-      <c r="I7" s="40" t="s">
+      <c r="H7" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="I7" s="39" t="s">
         <v>29</v>
       </c>
       <c r="J7" s="28" t="s">
@@ -2713,13 +2693,13 @@
     </row>
     <row r="8" s="1" customFormat="true" ht="69.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>9</v>
@@ -2734,7 +2714,7 @@
         <v>35</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>37</v>
@@ -2746,13 +2726,13 @@
     </row>
     <row r="9" s="1" customFormat="true" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>9</v>
@@ -2767,7 +2747,7 @@
         <v>35</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="I9" s="3" t="s">
         <v>37</v>
@@ -2779,13 +2759,13 @@
     </row>
     <row r="10" s="1" customFormat="true" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>9</v>
@@ -2800,7 +2780,7 @@
         <v>35</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="I10" s="3" t="s">
         <v>37</v>
@@ -2812,13 +2792,13 @@
     </row>
     <row r="11" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>9</v>
@@ -2833,23 +2813,23 @@
         <v>35</v>
       </c>
       <c r="H11" s="29" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="I11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J11" s="41"/>
+      <c r="J11" s="40"/>
       <c r="XEY11" s="0"/>
     </row>
     <row r="12" s="1" customFormat="true" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>9</v>
@@ -2860,172 +2840,172 @@
       <c r="F12" s="21" t="n">
         <v>46084</v>
       </c>
-      <c r="G12" s="42" t="s">
-        <v>113</v>
+      <c r="G12" s="41" t="s">
+        <v>133</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="J12" s="41"/>
+        <v>135</v>
+      </c>
+      <c r="J12" s="40"/>
       <c r="XEY12" s="0"/>
     </row>
     <row r="13" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="37"/>
+      <c r="A13" s="33"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="36"/>
       <c r="XEY13" s="0"/>
     </row>
     <row r="14" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="37"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="36"/>
       <c r="XEY14" s="0"/>
     </row>
     <row r="15" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="37"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="36"/>
       <c r="XEY15" s="0"/>
     </row>
     <row r="16" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="37"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="36"/>
       <c r="XEY16" s="0"/>
     </row>
     <row r="17" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="37"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="36"/>
       <c r="XEY17" s="0"/>
     </row>
     <row r="18" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="37"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="36"/>
       <c r="XEY18" s="0"/>
     </row>
     <row r="19" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="37"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="36"/>
       <c r="XEY19" s="0"/>
     </row>
     <row r="20" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="37"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="36"/>
       <c r="XEY20" s="0"/>
     </row>
     <row r="21" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="37"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="36"/>
       <c r="XEY21" s="0"/>
     </row>
     <row r="22" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="37"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="36"/>
       <c r="XEY22" s="0"/>
     </row>
     <row r="23" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="37"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="36"/>
       <c r="XEY23" s="0"/>
     </row>
     <row r="24" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="37"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="36"/>
       <c r="XEY24" s="0"/>
     </row>
     <row r="25" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="37"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="36"/>
       <c r="XEY25" s="0"/>
     </row>
   </sheetData>
@@ -3118,16 +3098,16 @@
         <v>24</v>
       </c>
       <c r="C7" s="20" t="s">
+        <v>136</v>
+      </c>
+      <c r="D7" s="20" t="s">
+        <v>137</v>
+      </c>
+      <c r="E7" s="20" t="s">
         <v>138</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="F7" s="20" t="s">
         <v>139</v>
-      </c>
-      <c r="E7" s="20" t="s">
-        <v>140</v>
-      </c>
-      <c r="F7" s="20" t="s">
-        <v>141</v>
       </c>
       <c r="G7" s="20" t="s">
         <v>27</v>
@@ -3144,31 +3124,31 @@
     </row>
     <row r="8" s="1" customFormat="true" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="E8" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="G8" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="H8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>146</v>
-      </c>
-      <c r="G8" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>148</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>37</v>
@@ -3176,31 +3156,31 @@
     </row>
     <row r="9" s="1" customFormat="true" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="G9" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I9" s="3" t="s">
         <v>153</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>155</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>37</v>
@@ -3208,31 +3188,31 @@
     </row>
     <row r="10" s="1" customFormat="true" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="E10" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="G10" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I10" s="3" t="s">
         <v>159</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G10" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>161</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>37</v>
@@ -3240,31 +3220,31 @@
     </row>
     <row r="11" s="1" customFormat="true" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C11" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="E11" s="3" t="s">
+      <c r="G11" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G11" s="22" t="s">
-        <v>147</v>
-      </c>
       <c r="H11" s="3" t="s">
         <v>37</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>37</v>
@@ -3272,31 +3252,31 @@
     </row>
     <row r="12" s="1" customFormat="true" ht="35.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="E12" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I12" s="3" t="s">
         <v>166</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="G12" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>168</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>37</v>
@@ -3304,31 +3284,31 @@
     </row>
     <row r="13" s="1" customFormat="true" ht="58.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="E13" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="D13" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="E13" s="3" t="s">
+      <c r="G13" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="F13" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G13" s="22" t="s">
-        <v>147</v>
-      </c>
       <c r="H13" s="3" t="s">
         <v>37</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>37</v>
@@ -3336,156 +3316,156 @@
     </row>
     <row r="14" s="1" customFormat="true" ht="46.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="E14" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G14" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="I14" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G14" s="22" t="s">
-        <v>147</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>176</v>
-      </c>
       <c r="J14" s="3" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="37"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="36"/>
     </row>
     <row r="16" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="37"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="36"/>
     </row>
     <row r="17" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="37"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="36"/>
     </row>
     <row r="18" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="37"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="36"/>
     </row>
     <row r="19" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="37"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="36"/>
     </row>
     <row r="20" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="37"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="36"/>
     </row>
     <row r="21" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="37"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="36"/>
     </row>
     <row r="22" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="37"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="36"/>
     </row>
     <row r="23" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="37"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="36"/>
     </row>
     <row r="24" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="37"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="36"/>
     </row>
     <row r="25" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="37"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
+      <c r="I25" s="36"/>
     </row>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3576,25 +3556,25 @@
         <v>23</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>24</v>
       </c>
       <c r="D7" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="F7" s="42" t="s">
         <v>178</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="G7" s="11" t="s">
         <v>179</v>
       </c>
-      <c r="F7" s="43" t="s">
+      <c r="H7" s="11" t="s">
         <v>180</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>182</v>
       </c>
       <c r="I7" s="11" t="s">
         <v>27</v>
@@ -3604,243 +3584,243 @@
       </c>
     </row>
     <row r="8" s="1" customFormat="true" ht="72.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="B8" s="44" t="s">
+      <c r="A8" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="43" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" s="43" t="s">
+        <v>182</v>
+      </c>
+      <c r="D8" s="44" t="s">
         <v>183</v>
       </c>
-      <c r="C8" s="44" t="s">
+      <c r="E8" s="45" t="s">
         <v>184</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="F8" s="46" t="s">
         <v>185</v>
       </c>
-      <c r="E8" s="46" t="s">
+      <c r="G8" s="46" t="s">
         <v>186</v>
       </c>
-      <c r="F8" s="47" t="s">
+      <c r="H8" s="44" t="s">
         <v>187</v>
       </c>
-      <c r="G8" s="47" t="s">
+      <c r="I8" s="47" t="s">
         <v>188</v>
       </c>
-      <c r="H8" s="45" t="s">
+      <c r="J8" s="48" t="s">
         <v>189</v>
       </c>
-      <c r="I8" s="48" t="s">
+    </row>
+    <row r="9" s="1" customFormat="true" ht="62.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="49" t="s">
+        <v>119</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" s="44" t="s">
         <v>190</v>
       </c>
-      <c r="J8" s="49" t="s">
+      <c r="D9" s="44" t="s">
+        <v>183</v>
+      </c>
+      <c r="E9" s="44" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="9" s="1" customFormat="true" ht="62.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="50" t="s">
-        <v>122</v>
-      </c>
-      <c r="B9" s="45" t="s">
-        <v>183</v>
-      </c>
-      <c r="C9" s="45" t="s">
+      <c r="F9" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="D9" s="45" t="s">
-        <v>185</v>
-      </c>
-      <c r="E9" s="45" t="s">
+      <c r="G9" s="46" t="s">
         <v>193</v>
       </c>
-      <c r="F9" s="51" t="s">
+      <c r="H9" s="44" t="s">
+        <v>187</v>
+      </c>
+      <c r="I9" s="47" t="s">
+        <v>188</v>
+      </c>
+      <c r="J9" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="G9" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="H9" s="45" t="s">
-        <v>189</v>
-      </c>
-      <c r="I9" s="48" t="s">
-        <v>190</v>
-      </c>
-      <c r="J9" s="29" t="s">
-        <v>196</v>
-      </c>
     </row>
     <row r="10" s="1" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="52"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="37"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="52"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="36"/>
     </row>
     <row r="11" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34"/>
-      <c r="B11" s="35"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="37"/>
+      <c r="A11" s="33"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="34"/>
+      <c r="F11" s="34"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="36"/>
     </row>
     <row r="12" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="37"/>
+      <c r="A12" s="33"/>
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+      <c r="D12" s="34"/>
+      <c r="E12" s="34"/>
+      <c r="F12" s="34"/>
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="36"/>
     </row>
     <row r="13" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="37"/>
+      <c r="A13" s="33"/>
+      <c r="B13" s="34"/>
+      <c r="C13" s="34"/>
+      <c r="D13" s="34"/>
+      <c r="E13" s="35"/>
+      <c r="F13" s="34"/>
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="36"/>
     </row>
     <row r="14" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="37"/>
+      <c r="A14" s="33"/>
+      <c r="B14" s="34"/>
+      <c r="C14" s="33"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="37"/>
+      <c r="I14" s="36"/>
     </row>
     <row r="15" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="37"/>
+      <c r="A15" s="33"/>
+      <c r="B15" s="33"/>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
+      <c r="E15" s="34"/>
+      <c r="F15" s="34"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="37"/>
+      <c r="I15" s="36"/>
     </row>
     <row r="16" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="37"/>
+      <c r="A16" s="33"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="34"/>
+      <c r="F16" s="34"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="37"/>
+      <c r="I16" s="36"/>
     </row>
     <row r="17" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="37"/>
+      <c r="A17" s="37"/>
+      <c r="B17" s="37"/>
+      <c r="C17" s="37"/>
+      <c r="D17" s="37"/>
+      <c r="E17" s="37"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="37"/>
+      <c r="H17" s="37"/>
+      <c r="I17" s="36"/>
     </row>
     <row r="18" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="37"/>
+      <c r="A18" s="37"/>
+      <c r="B18" s="37"/>
+      <c r="C18" s="37"/>
+      <c r="D18" s="37"/>
+      <c r="E18" s="37"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="37"/>
+      <c r="I18" s="36"/>
     </row>
     <row r="19" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="37"/>
+      <c r="A19" s="37"/>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="37"/>
+      <c r="I19" s="36"/>
     </row>
     <row r="20" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="37"/>
+      <c r="A20" s="37"/>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="36"/>
     </row>
     <row r="21" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="37"/>
+      <c r="A21" s="37"/>
+      <c r="B21" s="37"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="37"/>
+      <c r="E21" s="37"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="37"/>
+      <c r="H21" s="37"/>
+      <c r="I21" s="36"/>
     </row>
     <row r="22" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="37"/>
+      <c r="A22" s="37"/>
+      <c r="B22" s="37"/>
+      <c r="C22" s="37"/>
+      <c r="D22" s="37"/>
+      <c r="E22" s="37"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="37"/>
+      <c r="I22" s="36"/>
     </row>
     <row r="23" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="37"/>
+      <c r="A23" s="37"/>
+      <c r="B23" s="37"/>
+      <c r="C23" s="37"/>
+      <c r="D23" s="37"/>
+      <c r="E23" s="37"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="37"/>
+      <c r="H23" s="37"/>
+      <c r="I23" s="36"/>
     </row>
     <row r="24" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
+      <c r="A24" s="37"/>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="37"/>
+      <c r="E24" s="37"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="37"/>
       <c r="I24" s="8"/>
     </row>
     <row r="25" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
+      <c r="A25" s="37"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="37"/>
+      <c r="E25" s="37"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="37"/>
+      <c r="H25" s="37"/>
       <c r="I25" s="8"/>
     </row>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -3877,305 +3857,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A2:J1048576"/>
-  <sheetFormatPr defaultColWidth="9.2109375" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="8" width="20.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="8" width="33.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="8" width="35.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="8" width="31.7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="9" width="28.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="8" width="40.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="8" width="11.55"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="15" min="10" style="8" width="9.21"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16378" min="21" style="8" width="9.21"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16379" style="1" width="11.53"/>
-  </cols>
-  <sheetData>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="C2" s="13"/>
-    </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="13"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="13"/>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="16" t="n">
-        <v>46042</v>
-      </c>
-      <c r="C5" s="15"/>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="C7" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>178</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>179</v>
-      </c>
-      <c r="F7" s="43" t="s">
-        <v>180</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>181</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" s="1" customFormat="true" ht="23.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="9" s="1" customFormat="true" ht="25.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="10" s="1" customFormat="true" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="52"/>
-      <c r="B10" s="35"/>
-      <c r="C10" s="35"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="35"/>
-      <c r="F10" s="35"/>
-      <c r="G10" s="35"/>
-      <c r="H10" s="35"/>
-      <c r="I10" s="37"/>
-    </row>
-    <row r="11" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="34"/>
-      <c r="B11" s="35"/>
-      <c r="C11" s="34"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="35"/>
-      <c r="F11" s="35"/>
-      <c r="G11" s="35"/>
-      <c r="H11" s="35"/>
-      <c r="I11" s="37"/>
-    </row>
-    <row r="12" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="34"/>
-      <c r="B12" s="35"/>
-      <c r="C12" s="35"/>
-      <c r="D12" s="35"/>
-      <c r="E12" s="35"/>
-      <c r="F12" s="35"/>
-      <c r="G12" s="35"/>
-      <c r="H12" s="35"/>
-      <c r="I12" s="37"/>
-    </row>
-    <row r="13" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="34"/>
-      <c r="B13" s="35"/>
-      <c r="C13" s="35"/>
-      <c r="D13" s="35"/>
-      <c r="E13" s="36"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="35"/>
-      <c r="H13" s="35"/>
-      <c r="I13" s="37"/>
-    </row>
-    <row r="14" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="34"/>
-      <c r="B14" s="35"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="35"/>
-      <c r="E14" s="35"/>
-      <c r="F14" s="35"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="38"/>
-      <c r="I14" s="37"/>
-    </row>
-    <row r="15" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="34"/>
-      <c r="B15" s="34"/>
-      <c r="C15" s="34"/>
-      <c r="D15" s="34"/>
-      <c r="E15" s="35"/>
-      <c r="F15" s="35"/>
-      <c r="G15" s="35"/>
-      <c r="H15" s="38"/>
-      <c r="I15" s="37"/>
-    </row>
-    <row r="16" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34"/>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="35"/>
-      <c r="F16" s="35"/>
-      <c r="G16" s="35"/>
-      <c r="H16" s="38"/>
-      <c r="I16" s="37"/>
-    </row>
-    <row r="17" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38"/>
-      <c r="B17" s="38"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="38"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="38"/>
-      <c r="H17" s="38"/>
-      <c r="I17" s="37"/>
-    </row>
-    <row r="18" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38"/>
-      <c r="B18" s="38"/>
-      <c r="C18" s="38"/>
-      <c r="D18" s="38"/>
-      <c r="E18" s="38"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="37"/>
-      <c r="H18" s="38"/>
-      <c r="I18" s="37"/>
-    </row>
-    <row r="19" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38"/>
-      <c r="B19" s="38"/>
-      <c r="C19" s="38"/>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-      <c r="I19" s="37"/>
-    </row>
-    <row r="20" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38"/>
-      <c r="B20" s="38"/>
-      <c r="C20" s="38"/>
-      <c r="D20" s="38"/>
-      <c r="E20" s="38"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="37"/>
-      <c r="H20" s="38"/>
-      <c r="I20" s="37"/>
-    </row>
-    <row r="21" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38"/>
-      <c r="B21" s="38"/>
-      <c r="C21" s="38"/>
-      <c r="D21" s="38"/>
-      <c r="E21" s="38"/>
-      <c r="F21" s="39"/>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-      <c r="I21" s="37"/>
-    </row>
-    <row r="22" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="38"/>
-      <c r="B22" s="38"/>
-      <c r="C22" s="38"/>
-      <c r="D22" s="38"/>
-      <c r="E22" s="38"/>
-      <c r="F22" s="39"/>
-      <c r="G22" s="37"/>
-      <c r="H22" s="38"/>
-      <c r="I22" s="37"/>
-    </row>
-    <row r="23" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="38"/>
-      <c r="B23" s="38"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="38"/>
-      <c r="F23" s="39"/>
-      <c r="G23" s="38"/>
-      <c r="H23" s="38"/>
-      <c r="I23" s="37"/>
-    </row>
-    <row r="24" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38"/>
-      <c r="B24" s="38"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="37"/>
-      <c r="H24" s="38"/>
-      <c r="I24" s="8"/>
-    </row>
-    <row r="25" s="1" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="38"/>
-      <c r="B25" s="38"/>
-      <c r="C25" s="38"/>
-      <c r="D25" s="38"/>
-      <c r="E25" s="38"/>
-      <c r="F25" s="39"/>
-      <c r="G25" s="38"/>
-      <c r="H25" s="38"/>
-      <c r="I25" s="8"/>
-    </row>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-  </sheetData>
-  <conditionalFormatting sqref="I7">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>pass</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>failed</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="I1:I7 I24:I1007" type="list">
-      <formula1>"Pass ,Failed"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G10:G25" type="none">
-      <formula1>0</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="G26:G27" type="list">
-      <formula1>"Negative,Postive"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>